<commit_message>
Agregar plan de publicación en App Store y requisitos de iOS
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias de documentación/Matriz_de_Requisitos.xlsx
+++ b/Fase 2/Evidencias de documentación/Matriz_de_Requisitos.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Requisitos!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Requisitos!$A$4:$M$30</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Requisitos!$A$4:$M$32</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">'Requisitos técnicos'!$4:$4</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Resumen!$4:$4</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="320">
   <si>
     <t xml:space="preserve">Matriz de requisitos · Clancy's Rewards</t>
   </si>
@@ -405,6 +405,24 @@
     <t xml:space="preserve">HU-19</t>
   </si>
   <si>
+    <t xml:space="preserve">RF-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inicio de sesión con Apple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En iPhone, el cliente puede entrar con su cuenta de Apple, como alternativa al inicio de sesión con Google.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En la app de iOS aparece el botón "Iniciar sesión con Apple"; el servidor valida el token de Apple y crea o recupera la cuenta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guía de revisión de App Store 4.8 (por usar login con Google)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nueva HU-20 (publicación en App Store)</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNF-01</t>
   </si>
   <si>
@@ -564,16 +582,16 @@
     <t xml:space="preserve">Compatibilidad</t>
   </si>
   <si>
-    <t xml:space="preserve">App Android en Google Play</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La app se distribuye en Google Play, partiendo por una prueba cerrada.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La app pasa la prueba cerrada de 14 días con al menos 12 testers y queda publicada.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requisito de Google Play</t>
+    <t xml:space="preserve">App en Android e iOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La app se publica en Google Play y en App Store, con una sola base de código (Expo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android: pasa la prueba cerrada de 14 días con al menos 12 testers. iOS: el build de EAS pasa TestFlight y la revisión de Apple. Ambas quedan publicadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retroalimentación docente: el 47 % de los teléfonos en Irlanda usa iOS</t>
   </si>
   <si>
     <t xml:space="preserve">Sprint 2 y cierre</t>
@@ -582,7 +600,7 @@
     <t xml:space="preserve">#51</t>
   </si>
   <si>
-    <t xml:space="preserve">Issues #51, #53 y #60</t>
+    <t xml:space="preserve">Issues #51, #53 y #60, más las tareas de iOS</t>
   </si>
   <si>
     <t xml:space="preserve">RNF-10</t>
@@ -630,6 +648,24 @@
     <t xml:space="preserve">Issues #58 y #59</t>
   </si>
   <si>
+    <t xml:space="preserve">RNF-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requisitos de publicación en App Store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La app cumple las reglas de Apple: texto de permiso de cámara, política de privacidad, etiqueta de privacidad y borrado de cuenta dentro de la app.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La ficha de App Store está completa y la app no es rechazada en la revisión por estos puntos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guía de revisión de App Store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ficha de App Store y app.json</t>
+  </si>
+  <si>
     <t xml:space="preserve">Leyenda: Estado y Prioridad se eligen de una lista. El estado se actualiza al cerrar el issue de cada requisito; el resumen se recalcula solo.</t>
   </si>
   <si>
@@ -897,16 +933,61 @@
     <t xml:space="preserve">Dirección propia para la API</t>
   </si>
   <si>
-    <t xml:space="preserve">EAS Build (Expo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compilar la app de producción para Google Play</t>
+    <t xml:space="preserve">EAS Build y EAS Submit (Expo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan gratuito: hasta 15 builds iOS y 15 Android al mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compilar la app en la nube para Android e iOS, sin necesidad de un Mac, y enviarla a las tiendas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apple Developer Program</t>
+  </si>
+  <si>
+    <t xml:space="preserve">99 USD al año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuenta de desarrollador para TestFlight y App Store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestFlight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incluido en la cuenta de Apple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prueba de la app de iOS con iPhones reales antes de publicar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mac en la nube (MacinCloud), solo si hace falta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desde 1 USD por hora, prepago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Respaldo si un error de iOS necesita Xcode; no es necesario para compilar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iPhone de prueba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prestado o de testers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probar la app de iOS con TestFlight (personal del local y conocidos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">expo-apple-authentication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inicio de sesión con Apple en iOS</t>
   </si>
   <si>
     <t xml:space="preserve">Costo total estimado del proyecto</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuente de los costos: documento de definición del proyecto (Fase 1). Las versiones salen de package.json y requirements.txt del repositorio.</t>
+    <t xml:space="preserve">Fuentes de los costos: documento de definición del proyecto (Fase 1); Apple Developer Program (developer.apple.com); planes de Expo (expo.dev/pricing); MacinCloud (macincloud.com). Las versiones salen de package.json y requirements.txt.</t>
   </si>
 </sst>
 </file>
@@ -1483,7 +1564,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -2173,63 +2254,63 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>125</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>129</v>
-      </c>
       <c r="F20" s="5" t="s">
-        <v>130</v>
+        <v>20</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>24</v>
+        <v>93</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="L20" s="6"/>
       <c r="M20" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="F21" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>130</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>21</v>
@@ -2238,7 +2319,7 @@
         <v>137</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>24</v>
@@ -2248,36 +2329,36 @@
       </c>
       <c r="L21" s="6"/>
       <c r="M21" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>24</v>
@@ -2287,83 +2368,81 @@
       </c>
       <c r="L22" s="6"/>
       <c r="M22" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>24</v>
       </c>
       <c r="K23" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L23" s="6"/>
+      <c r="M23" s="5" t="s">
         <v>149</v>
-      </c>
-      <c r="L23" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="M23" s="5" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>154</v>
-      </c>
       <c r="F24" s="5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H24" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K24" s="6" t="s">
         <v>155</v>
-      </c>
-      <c r="I24" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="J24" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="L24" s="7" t="s">
         <v>156</v>
@@ -2377,10 +2456,10 @@
         <v>158</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>88</v>
+        <v>133</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>159</v>
@@ -2389,16 +2468,16 @@
         <v>160</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>72</v>
+        <v>136</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>161</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>92</v>
+        <v>138</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>93</v>
@@ -2418,221 +2497,301 @@
         <v>164</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C26" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="F26" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H26" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="F26" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>168</v>
-      </c>
       <c r="I26" s="5" t="s">
-        <v>169</v>
+        <v>92</v>
       </c>
       <c r="J26" s="6" t="s">
         <v>93</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>33</v>
+        <v>94</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="D27" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="E27" s="5" t="s">
-        <v>174</v>
-      </c>
       <c r="F27" s="5" t="s">
-        <v>20</v>
+        <v>136</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H27" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="I27" s="5" t="s">
         <v>175</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>122</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>93</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>107</v>
+        <v>33</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>124</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>177</v>
+        <v>118</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>130</v>
+        <v>20</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>181</v>
+        <v>122</v>
       </c>
       <c r="J28" s="6" t="s">
         <v>93</v>
       </c>
       <c r="K28" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="L28" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="M28" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="L28" s="7" t="s">
+      <c r="B29" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="M28" s="5" t="s">
+      <c r="D29" s="5" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+      <c r="E29" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C29" s="5" t="s">
+      <c r="F29" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H29" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="I29" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="J29" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="K29" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="F29" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="H29" s="5" t="s">
+      <c r="L29" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="I29" s="5" t="s">
+      <c r="M29" s="5" t="s">
         <v>190</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L29" s="6"/>
-      <c r="M29" s="5" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C30" s="5" t="s">
+      <c r="D30" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="E30" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="F30" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H30" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="F30" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="G30" s="6" t="s">
+      <c r="I30" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L30" s="6"/>
+      <c r="M30" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="G31" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H30" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="I30" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="J30" s="6" t="s">
+      <c r="H31" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="J31" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="K30" s="6" t="s">
+      <c r="K31" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="L30" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="M30" s="5" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="s">
-        <v>201</v>
+      <c r="L31" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="M31" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="L32" s="6"/>
+      <c r="M32" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M30"/>
+  <autoFilter ref="A4:M32"/>
   <mergeCells count="2">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J5:J30">
+  <conditionalFormatting sqref="J5:J32">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$J5="Implementado"</formula>
     </cfRule>
@@ -2644,11 +2803,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J30" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J32" type="list">
       <formula1>"Implementado,Parcial,Pendiente"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G30" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G32" type="list">
       <formula1>"Alta,Media,Baja"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2660,13 +2819,13 @@
     <hyperlink ref="L17" r:id="rId4" display="#57"/>
     <hyperlink ref="L18" r:id="rId5" display="#56"/>
     <hyperlink ref="L19" r:id="rId6" display="#54"/>
-    <hyperlink ref="L23" r:id="rId7" display="#36"/>
-    <hyperlink ref="L24" r:id="rId8" display="#42"/>
-    <hyperlink ref="L25" r:id="rId9" display="#45"/>
-    <hyperlink ref="L26" r:id="rId10" display="#47"/>
-    <hyperlink ref="L27" r:id="rId11" display="#54"/>
-    <hyperlink ref="L28" r:id="rId12" display="#51"/>
-    <hyperlink ref="L30" r:id="rId13" display="#58"/>
+    <hyperlink ref="L24" r:id="rId7" display="#36"/>
+    <hyperlink ref="L25" r:id="rId8" display="#42"/>
+    <hyperlink ref="L26" r:id="rId9" display="#45"/>
+    <hyperlink ref="L27" r:id="rId10" display="#47"/>
+    <hyperlink ref="L28" r:id="rId11" display="#54"/>
+    <hyperlink ref="L29" r:id="rId12" display="#51"/>
+    <hyperlink ref="L31" r:id="rId13" display="#58"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2697,7 +2856,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2707,7 +2866,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2720,7 +2879,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>24</v>
@@ -2732,7 +2891,7 @@
         <v>93</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2740,58 +2899,58 @@
         <v>16</v>
       </c>
       <c r="B5" s="10" t="n">
-        <f aca="false">COUNTIF(Requisitos!$B$5:$B$30,A5)</f>
-        <v>15</v>
+        <f aca="false">COUNTIF(Requisitos!$B$5:$B$32,A5)</f>
+        <v>16</v>
       </c>
       <c r="C5" s="10" t="n">
-        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$30,A5,Requisitos!$J$5:$J$30,"Implementado")</f>
+        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A5,Requisitos!$J$5:$J$32,"Implementado")</f>
         <v>9</v>
       </c>
       <c r="D5" s="10" t="n">
-        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$30,A5,Requisitos!$J$5:$J$30,"Parcial")</f>
+        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A5,Requisitos!$J$5:$J$32,"Parcial")</f>
         <v>1</v>
       </c>
       <c r="E5" s="10" t="n">
-        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$30,A5,Requisitos!$J$5:$J$30,"Pendiente")</f>
-        <v>5</v>
+        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A5,Requisitos!$J$5:$J$32,"Pendiente")</f>
+        <v>6</v>
       </c>
       <c r="F5" s="11" t="n">
         <f aca="false">IF(B5=0,0,C5/B5)</f>
-        <v>0.6</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">COUNTIF(Requisitos!$B$5:$B$30,A6)</f>
-        <v>11</v>
+        <f aca="false">COUNTIF(Requisitos!$B$5:$B$32,A6)</f>
+        <v>12</v>
       </c>
       <c r="C6" s="10" t="n">
-        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$30,A6,Requisitos!$J$5:$J$30,"Implementado")</f>
+        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A6,Requisitos!$J$5:$J$32,"Implementado")</f>
         <v>5</v>
       </c>
       <c r="D6" s="10" t="n">
-        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$30,A6,Requisitos!$J$5:$J$30,"Parcial")</f>
+        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A6,Requisitos!$J$5:$J$32,"Parcial")</f>
         <v>0</v>
       </c>
       <c r="E6" s="10" t="n">
-        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$30,A6,Requisitos!$J$5:$J$30,"Pendiente")</f>
-        <v>6</v>
+        <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A6,Requisitos!$J$5:$J$32,"Pendiente")</f>
+        <v>7</v>
       </c>
       <c r="F6" s="11" t="n">
         <f aca="false">IF(B6=0,0,C6/B6)</f>
-        <v>0.454545454545455</v>
+        <v>0.416666666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">SUM(B5:B6)</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7" s="13" t="n">
         <f aca="false">SUM(C5:C6)</f>
@@ -2803,11 +2962,11 @@
       </c>
       <c r="E7" s="13" t="n">
         <f aca="false">SUM(E5:E6)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F7" s="14" t="n">
         <f aca="false">IF(B7=0,0,C7/B7)</f>
-        <v>0.538461538461538</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2815,7 +2974,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2823,16 +2982,16 @@
         <v>25</v>
       </c>
       <c r="B10" s="10" t="n">
-        <f aca="false">COUNTIF(Requisitos!$K$5:$K$30,"Prototipo*")</f>
+        <f aca="false">COUNTIF(Requisitos!$K$5:$K$32,"Prototipo*")</f>
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">COUNTIF(Requisitos!$K$5:$K$30,"Sprint 0*")</f>
+        <f aca="false">COUNTIF(Requisitos!$K$5:$K$32,"Sprint 0*")</f>
         <v>1</v>
       </c>
     </row>
@@ -2841,7 +3000,7 @@
         <v>94</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">COUNTIF(Requisitos!$K$5:$K$30,"Sprint 1*")</f>
+        <f aca="false">COUNTIF(Requisitos!$K$5:$K$32,"Sprint 1*")</f>
         <v>4</v>
       </c>
     </row>
@@ -2850,8 +3009,8 @@
         <v>33</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">COUNTIF(Requisitos!$K$5:$K$30,"Sprint 2*")</f>
-        <v>3</v>
+        <f aca="false">COUNTIF(Requisitos!$K$5:$K$32,"Sprint 2*")</f>
+        <v>4</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2859,13 +3018,13 @@
         <v>107</v>
       </c>
       <c r="B14" s="10" t="n">
-        <f aca="false">COUNTIF(Requisitos!$K$5:$K$30,"Sprint 3*")</f>
-        <v>5</v>
+        <f aca="false">COUNTIF(Requisitos!$K$5:$K$32,"Sprint 3*")</f>
+        <v>6</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -2888,7 +3047,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -2900,7 +3059,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2910,7 +3069,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2920,36 +3079,36 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="E5" s="17" t="n">
         <v>0</v>
@@ -2960,16 +3119,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>0</v>
@@ -2980,16 +3139,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>0</v>
@@ -3000,16 +3159,16 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>0</v>
@@ -3020,16 +3179,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>0</v>
@@ -3040,16 +3199,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>0</v>
@@ -3060,16 +3219,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="E11" s="17" t="n">
         <v>0</v>
@@ -3080,16 +3239,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>0</v>
@@ -3100,16 +3259,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="E13" s="17" t="n">
         <v>0</v>
@@ -3120,16 +3279,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>0</v>
@@ -3140,16 +3299,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="E15" s="17" t="n">
         <v>0</v>
@@ -3160,16 +3319,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>0</v>
@@ -3180,16 +3339,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="E17" s="17" t="n">
         <v>0</v>
@@ -3200,16 +3359,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="E18" s="17" t="n">
         <v>0</v>
@@ -3220,16 +3379,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="E19" s="17" t="n">
         <v>0</v>
@@ -3240,16 +3399,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="E20" s="17" t="n">
         <v>0</v>
@@ -3260,16 +3419,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="E21" s="17" t="n">
         <v>0</v>
@@ -3280,16 +3439,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="E22" s="17" t="n">
         <v>0</v>
@@ -3300,16 +3459,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="E23" s="17" t="n">
         <v>0</v>
@@ -3320,16 +3479,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="E24" s="17" t="n">
         <v>25</v>
@@ -3340,16 +3499,16 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="E25" s="17" t="n">
         <v>0</v>
@@ -3360,16 +3519,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="E26" s="17" t="n">
         <v>0</v>
@@ -3380,16 +3539,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="E27" s="17" t="n">
         <v>10</v>
@@ -3398,18 +3557,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>276</v>
+        <v>302</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="E28" s="17" t="n">
         <v>0</v>
@@ -3419,24 +3578,124 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18"/>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="19" t="s">
-        <v>291</v>
-      </c>
-      <c r="E29" s="20" t="n">
-        <f aca="false">SUM(E5:E28)</f>
-        <v>35</v>
-      </c>
-      <c r="F29" s="20" t="n">
-        <f aca="false">SUM(F5:F28)</f>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="s">
-        <v>292</v>
+      <c r="A29" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="E29" s="17" t="n">
+        <v>99</v>
+      </c>
+      <c r="F29" s="17" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="E30" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>310</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E31" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="17" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="E32" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="E33" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="E34" s="20" t="n">
+        <f aca="false">SUM(E5:E33)</f>
+        <v>134</v>
+      </c>
+      <c r="F34" s="20" t="n">
+        <f aca="false">SUM(F5:F33)</f>
+        <v>183</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="s">
+        <v>319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enlazar los requisitos y el plan de iOS con sus issues
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias de documentación/Matriz_de_Requisitos.xlsx
+++ b/Fase 2/Evidencias de documentación/Matriz_de_Requisitos.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="322">
   <si>
     <t xml:space="preserve">Matriz de requisitos · Clancy's Rewards</t>
   </si>
@@ -420,7 +420,10 @@
     <t xml:space="preserve">Guía de revisión de App Store 4.8 (por usar login con Google)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nueva HU-20 (publicación en App Store)</t>
+    <t xml:space="preserve">#66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-20</t>
   </si>
   <si>
     <t xml:space="preserve">RNF-01</t>
@@ -600,7 +603,7 @@
     <t xml:space="preserve">#51</t>
   </si>
   <si>
-    <t xml:space="preserve">Issues #51, #53 y #60, más las tareas de iOS</t>
+    <t xml:space="preserve">Android: #51, #53 y #60 · iOS: #65, #67, #69 y #70</t>
   </si>
   <si>
     <t xml:space="preserve">RNF-10</t>
@@ -663,7 +666,10 @@
     <t xml:space="preserve">Guía de revisión de App Store</t>
   </si>
   <si>
-    <t xml:space="preserve">Ficha de App Store y app.json</t>
+    <t xml:space="preserve">#68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Issues #68 y #70</t>
   </si>
   <si>
     <t xml:space="preserve">Leyenda: Estado y Prioridad se eligen de una lista. El estado se actualiza al cerrar el issue de cada requisito; el resumen se recalcula solo.</t>
@@ -2288,38 +2294,40 @@
       <c r="K20" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="L20" s="6"/>
+      <c r="L20" s="7" t="s">
+        <v>130</v>
+      </c>
       <c r="M20" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>24</v>
@@ -2329,36 +2337,36 @@
       </c>
       <c r="L21" s="6"/>
       <c r="M21" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>24</v>
@@ -2368,36 +2376,36 @@
       </c>
       <c r="L22" s="6"/>
       <c r="M22" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>24</v>
@@ -2407,77 +2415,77 @@
       </c>
       <c r="L23" s="6"/>
       <c r="M23" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>24</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>93</v>
@@ -2486,27 +2494,27 @@
         <v>94</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>88</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>72</v>
@@ -2515,7 +2523,7 @@
         <v>65</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>92</v>
@@ -2527,39 +2535,39 @@
         <v>94</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>93</v>
@@ -2568,27 +2576,27 @@
         <v>33</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>118</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F28" s="5" t="s">
         <v>20</v>
@@ -2597,7 +2605,7 @@
         <v>21</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>122</v>
@@ -2617,60 +2625,60 @@
     </row>
     <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J29" s="6" t="s">
         <v>93</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>72</v>
@@ -2679,10 +2687,10 @@
         <v>65</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J30" s="6" t="s">
         <v>24</v>
@@ -2692,36 +2700,36 @@
       </c>
       <c r="L30" s="6"/>
       <c r="M30" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J31" s="6" t="s">
         <v>93</v>
@@ -2730,39 +2738,39 @@
         <v>107</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J32" s="6" t="s">
         <v>93</v>
@@ -2770,19 +2778,21 @@
       <c r="K32" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="L32" s="6"/>
+      <c r="L32" s="7" t="s">
+        <v>212</v>
+      </c>
       <c r="M32" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -2819,13 +2829,15 @@
     <hyperlink ref="L17" r:id="rId4" display="#57"/>
     <hyperlink ref="L18" r:id="rId5" display="#56"/>
     <hyperlink ref="L19" r:id="rId6" display="#54"/>
-    <hyperlink ref="L24" r:id="rId7" display="#36"/>
-    <hyperlink ref="L25" r:id="rId8" display="#42"/>
-    <hyperlink ref="L26" r:id="rId9" display="#45"/>
-    <hyperlink ref="L27" r:id="rId10" display="#47"/>
-    <hyperlink ref="L28" r:id="rId11" display="#54"/>
-    <hyperlink ref="L29" r:id="rId12" display="#51"/>
-    <hyperlink ref="L31" r:id="rId13" display="#58"/>
+    <hyperlink ref="L20" r:id="rId7" display="#66"/>
+    <hyperlink ref="L24" r:id="rId8" display="#36"/>
+    <hyperlink ref="L25" r:id="rId9" display="#42"/>
+    <hyperlink ref="L26" r:id="rId10" display="#45"/>
+    <hyperlink ref="L27" r:id="rId11" display="#47"/>
+    <hyperlink ref="L28" r:id="rId12" display="#54"/>
+    <hyperlink ref="L29" r:id="rId13" display="#51"/>
+    <hyperlink ref="L31" r:id="rId14" display="#58"/>
+    <hyperlink ref="L32" r:id="rId15" display="#68"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2834,7 +2846,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId14"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
 
@@ -2856,7 +2868,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2866,7 +2878,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2879,7 +2891,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>24</v>
@@ -2891,7 +2903,7 @@
         <v>93</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2921,7 +2933,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">COUNTIF(Requisitos!$B$5:$B$32,A6)</f>
@@ -2946,7 +2958,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">SUM(B5:B6)</f>
@@ -2974,7 +2986,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2988,7 +3000,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">COUNTIF(Requisitos!$K$5:$K$32,"Sprint 0*")</f>
@@ -3024,7 +3036,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -3059,7 +3071,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3069,7 +3081,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3079,36 +3091,36 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E5" s="17" t="n">
         <v>0</v>
@@ -3119,16 +3131,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B6" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>230</v>
-      </c>
       <c r="D6" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>0</v>
@@ -3139,16 +3151,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>0</v>
@@ -3159,16 +3171,16 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>0</v>
@@ -3179,16 +3191,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>0</v>
@@ -3199,16 +3211,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>0</v>
@@ -3219,16 +3231,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E11" s="17" t="n">
         <v>0</v>
@@ -3239,16 +3251,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>0</v>
@@ -3259,16 +3271,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E13" s="17" t="n">
         <v>0</v>
@@ -3279,16 +3291,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>0</v>
@@ -3299,16 +3311,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E15" s="17" t="n">
         <v>0</v>
@@ -3319,16 +3331,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>0</v>
@@ -3339,16 +3351,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E17" s="17" t="n">
         <v>0</v>
@@ -3359,16 +3371,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E18" s="17" t="n">
         <v>0</v>
@@ -3379,16 +3391,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E19" s="17" t="n">
         <v>0</v>
@@ -3399,16 +3411,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E20" s="17" t="n">
         <v>0</v>
@@ -3419,16 +3431,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E21" s="17" t="n">
         <v>0</v>
@@ -3439,16 +3451,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E22" s="17" t="n">
         <v>0</v>
@@ -3459,16 +3471,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E23" s="17" t="n">
         <v>0</v>
@@ -3479,16 +3491,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E24" s="17" t="n">
         <v>25</v>
@@ -3499,16 +3511,16 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E25" s="17" t="n">
         <v>0</v>
@@ -3519,16 +3531,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E26" s="17" t="n">
         <v>0</v>
@@ -3539,16 +3551,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E27" s="17" t="n">
         <v>10</v>
@@ -3559,16 +3571,16 @@
     </row>
     <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E28" s="17" t="n">
         <v>0</v>
@@ -3579,16 +3591,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E29" s="17" t="n">
         <v>99</v>
@@ -3599,16 +3611,16 @@
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E30" s="17" t="n">
         <v>0</v>
@@ -3619,16 +3631,16 @@
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E31" s="17" t="n">
         <v>0</v>
@@ -3639,16 +3651,16 @@
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E32" s="17" t="n">
         <v>0</v>
@@ -3659,16 +3671,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>318</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="B33" s="16" t="s">
-        <v>316</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>242</v>
-      </c>
       <c r="D33" s="5" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="E33" s="17" t="n">
         <v>0</v>
@@ -3682,7 +3694,7 @@
       <c r="B34" s="18"/>
       <c r="C34" s="18"/>
       <c r="D34" s="19" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E34" s="20" t="n">
         <f aca="false">SUM(E5:E33)</f>
@@ -3695,7 +3707,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar el avance del Sprint 1: CORS, límite de intentos y primeras pruebas
- Matriz de requisitos: RNF-05 implementado y RNF-11 parcial, con su evidencia.
- Informe de avance: fecha de corte 29 de octubre, estado del Sprint 1 y de las pruebas.
- Presentación: RNF-05 listo y línea de avance del Sprint 1.
- Arquitectura y README: seguridad aplicada y cómo correr las pruebas.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias de documentación/Matriz_de_Requisitos.xlsx
+++ b/Fase 2/Evidencias de documentación/Matriz_de_Requisitos.xlsx
@@ -33,7 +33,7 @@
     <t xml:space="preserve">Matriz de requisitos · Clancy's Rewards</t>
   </si>
   <si>
-    <t xml:space="preserve">Capstone 001V · Andy Aravena Auquilen · Estado al 28 de octubre de 2026</t>
+    <t xml:space="preserve">Capstone 001V · Andy Aravena Auquilen · Estado al 29 de octubre de 2026</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -516,13 +516,13 @@
     <t xml:space="preserve">Se limitan los intentos de login y de escaneo, y la API solo acepta orígenes conocidos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tras varios intentos fallidos la API responde error 429; un origen no autorizado es rechazado.</t>
+    <t xml:space="preserve">Tras 5 intentos fallidos de login en 15 minutos, o más de 20 escaneos por minuto, la API responde error 429; un origen que no está en CORS_ORIGINS es rechazado.</t>
   </si>
   <si>
     <t xml:space="preserve">#42</t>
   </si>
   <si>
-    <t xml:space="preserve">Issues #41 y #42</t>
+    <t xml:space="preserve">backend/server.py · backend/tests/test_limite_intentos.py · Issues #41 y #42</t>
   </si>
   <si>
     <t xml:space="preserve">RNF-06</t>
@@ -648,7 +648,7 @@
     <t xml:space="preserve">#58</t>
   </si>
   <si>
-    <t xml:space="preserve">Issues #58 y #59</t>
+    <t xml:space="preserve">backend/tests (10 pruebas del límite de intentos) · Issues #58 y #59</t>
   </si>
   <si>
     <t xml:space="preserve">RNF-12</t>
@@ -2459,7 +2459,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
         <v>159</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>139</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="K25" s="6" t="s">
         <v>94</v>
@@ -2732,7 +2732,7 @@
         <v>204</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>93</v>
+        <v>32</v>
       </c>
       <c r="K31" s="6" t="s">
         <v>107</v>
@@ -2941,19 +2941,19 @@
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A6,Requisitos!$J$5:$J$32,"Implementado")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="10" t="n">
         <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A6,Requisitos!$J$5:$J$32,"Parcial")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">COUNTIFS(Requisitos!$B$5:$B$32,A6,Requisitos!$J$5:$J$32,"Pendiente")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F6" s="11" t="n">
         <f aca="false">IF(B6=0,0,C6/B6)</f>
-        <v>0.416666666666667</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2966,19 +2966,19 @@
       </c>
       <c r="C7" s="13" t="n">
         <f aca="false">SUM(C5:C6)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" s="13" t="n">
         <f aca="false">SUM(D5:D6)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" s="13" t="n">
         <f aca="false">SUM(E5:E6)</f>
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F7" s="14" t="n">
         <f aca="false">IF(B7=0,0,C7/B7)</f>
-        <v>0.5</v>
+        <v>0.535714285714286</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>